<commit_message>
added and remove the files
</commit_message>
<xml_diff>
--- a/attendence_summary.xlsx
+++ b/attendence_summary.xlsx
@@ -463,7 +463,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -471,11 +471,11 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>3.827083333333333</v>
+        <v>8.720833333333333</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>91:51</t>
+          <t>209:18</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -494,11 +494,11 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0</v>
+        <v>8.740277777777777</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>209:46</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -517,11 +517,11 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>5.651388888888889</v>
+        <v>8.184027777777779</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>135:38</t>
+          <t>196:25</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -540,11 +540,11 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>2.859722222222222</v>
+        <v>5.64375</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>68:38</t>
+          <t>135:27</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -563,11 +563,11 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0</v>
+        <v>7.319444444444445</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>175:40</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -586,11 +586,11 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>5.040972222222222</v>
+        <v>8.875694444444445</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>120:59</t>
+          <t>213:01</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -609,11 +609,11 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0</v>
+        <v>7.728472222222222</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>185:29</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -632,11 +632,11 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0</v>
+        <v>7.728472222222222</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>185:29</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -655,11 +655,11 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0</v>
+        <v>7.728472222222222</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>185:29</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -678,11 +678,11 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0</v>
+        <v>7.728472222222222</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>185:29</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -701,11 +701,11 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>1.957638888888889</v>
+        <v>5.632638888888889</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>46:59</t>
+          <t>135:11</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -724,11 +724,11 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>2.313888888888889</v>
+        <v>5.233333333333333</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>55:32</t>
+          <t>125:36</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -747,11 +747,11 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>2.5875</v>
+        <v>5.870138888888889</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>62:06</t>
+          <t>140:53</t>
         </is>
       </c>
     </row>
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -770,11 +770,11 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>1.943055555555556</v>
+        <v>5.935416666666667</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>46:38</t>
+          <t>142:27</t>
         </is>
       </c>
     </row>
@@ -785,7 +785,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -793,11 +793,11 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0</v>
+        <v>3.272222222222222</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>78:32</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -816,11 +816,11 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0</v>
+        <v>3.272222222222222</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>78:32</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -839,11 +839,11 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>3.886805555555556</v>
+        <v>5.674305555555556</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>93:17</t>
+          <t>136:11</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -862,11 +862,11 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.5604166666666667</v>
+        <v>5.311111111111111</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>13:27</t>
+          <t>127:28</t>
         </is>
       </c>
     </row>
@@ -877,7 +877,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -885,11 +885,11 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>3.188888888888889</v>
+        <v>4.49375</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>76:32</t>
+          <t>107:51</t>
         </is>
       </c>
     </row>
@@ -900,7 +900,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -908,11 +908,11 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>3.054166666666667</v>
+        <v>5.26875</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>73:18</t>
+          <t>126:27</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -931,11 +931,11 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0</v>
+        <v>6.329166666666667</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>151:54</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -954,11 +954,11 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>1.022916666666667</v>
+        <v>3.950694444444444</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>24:33</t>
+          <t>94:49</t>
         </is>
       </c>
     </row>
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -977,11 +977,11 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>4.13125</v>
+        <v>7.559722222222222</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>99:09</t>
+          <t>181:26</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1000,11 +1000,11 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.3590277777777778</v>
+        <v>5.938194444444444</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>08:37</t>
+          <t>142:31</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1023,11 +1023,11 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0.4805555555555556</v>
+        <v>3.472222222222222</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>11:32</t>
+          <t>83:20</t>
         </is>
       </c>
     </row>

</xml_diff>